<commit_message>
Table A7: replace per-cell N with count meeting each streak definition
N was constant (2,214) in every cell by construction -- the streak
indicator is never missing, so it never changes which rows survive the
complete-case filter. Reporting it once per cell was redundant; the
manuscript's Table A7 already states N=2,214 once in the notes.
Replaced with the more informative raw count of observations meeting
each streak definition (already available in
h3_bar_sensitivity_coverage.csv, alongside the % column). No
coefficient, SE, p-value, or the underlying N itself changed --
presentation only.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/tableA7_h3_bar_sensitivity.xlsx
+++ b/results/tables/tableA7_h3_bar_sensitivity.xlsx
@@ -31,7 +31,7 @@
     <t>streak_ge24_p</t>
   </si>
   <si>
-    <t>streak_ge24_n</t>
+    <t>streak_ge24_count_meeting</t>
   </si>
   <si>
     <t>streak_ge24_pct_meeting</t>
@@ -46,7 +46,7 @@
     <t>streak_ge36_p</t>
   </si>
   <si>
-    <t>streak_ge36_n</t>
+    <t>streak_ge36_count_meeting</t>
   </si>
   <si>
     <t>streak_ge36_pct_meeting</t>
@@ -61,7 +61,7 @@
     <t>streak_ge60_p</t>
   </si>
   <si>
-    <t>streak_ge60_n</t>
+    <t>streak_ge60_count_meeting</t>
   </si>
   <si>
     <t>streak_ge60_pct_meeting</t>
@@ -495,7 +495,7 @@
         <v>0.4701406943915962</v>
       </c>
       <c r="F2">
-        <v>2214</v>
+        <v>864</v>
       </c>
       <c r="G2">
         <v>39</v>
@@ -510,7 +510,7 @@
         <v>0.0323195934941913</v>
       </c>
       <c r="K2">
-        <v>2214</v>
+        <v>756</v>
       </c>
       <c r="L2">
         <v>34.1</v>
@@ -525,7 +525,7 @@
         <v>0.0053930115768539</v>
       </c>
       <c r="P2">
-        <v>2214</v>
+        <v>598</v>
       </c>
       <c r="Q2">
         <v>27</v>
@@ -548,7 +548,7 @@
         <v>0.07259079469274771</v>
       </c>
       <c r="F3">
-        <v>2214</v>
+        <v>693</v>
       </c>
       <c r="G3">
         <v>31.3</v>
@@ -563,7 +563,7 @@
         <v>0.0426184093047121</v>
       </c>
       <c r="K3">
-        <v>2214</v>
+        <v>600</v>
       </c>
       <c r="L3">
         <v>27.1</v>
@@ -578,7 +578,7 @@
         <v>0.06863983200403</v>
       </c>
       <c r="P3">
-        <v>2214</v>
+        <v>469</v>
       </c>
       <c r="Q3">
         <v>21.2</v>
@@ -601,7 +601,7 @@
         <v>0.0155021492672648</v>
       </c>
       <c r="F4">
-        <v>2214</v>
+        <v>599</v>
       </c>
       <c r="G4">
         <v>27.1</v>
@@ -616,7 +616,7 @@
         <v>0.007954422130128201</v>
       </c>
       <c r="K4">
-        <v>2214</v>
+        <v>516</v>
       </c>
       <c r="L4">
         <v>23.3</v>
@@ -631,7 +631,7 @@
         <v>0.0441753969838323</v>
       </c>
       <c r="P4">
-        <v>2214</v>
+        <v>405</v>
       </c>
       <c r="Q4">
         <v>18.3</v>
@@ -654,7 +654,7 @@
         <v>0.0912766669107223</v>
       </c>
       <c r="F5">
-        <v>2214</v>
+        <v>513</v>
       </c>
       <c r="G5">
         <v>23.2</v>
@@ -669,7 +669,7 @@
         <v>0.0909708280126286</v>
       </c>
       <c r="K5">
-        <v>2214</v>
+        <v>438</v>
       </c>
       <c r="L5">
         <v>19.8</v>
@@ -684,7 +684,7 @@
         <v>0.09552491846392171</v>
       </c>
       <c r="P5">
-        <v>2214</v>
+        <v>339</v>
       </c>
       <c r="Q5">
         <v>15.3</v>
@@ -707,7 +707,7 @@
         <v>0.0387679259308531</v>
       </c>
       <c r="F6">
-        <v>2214</v>
+        <v>452</v>
       </c>
       <c r="G6">
         <v>20.4</v>
@@ -722,7 +722,7 @@
         <v>0.1171568912763221</v>
       </c>
       <c r="K6">
-        <v>2214</v>
+        <v>386</v>
       </c>
       <c r="L6">
         <v>17.4</v>
@@ -737,7 +737,7 @@
         <v>0.0974813766091613</v>
       </c>
       <c r="P6">
-        <v>2214</v>
+        <v>296</v>
       </c>
       <c r="Q6">
         <v>13.4</v>
@@ -760,7 +760,7 @@
         <v>0.0896835702361045</v>
       </c>
       <c r="F7">
-        <v>2214</v>
+        <v>292</v>
       </c>
       <c r="G7">
         <v>13.2</v>
@@ -775,7 +775,7 @@
         <v>0.5823129729668779</v>
       </c>
       <c r="K7">
-        <v>2214</v>
+        <v>242</v>
       </c>
       <c r="L7">
         <v>10.9</v>
@@ -790,7 +790,7 @@
         <v>0.8156224085271169</v>
       </c>
       <c r="P7">
-        <v>2214</v>
+        <v>186</v>
       </c>
       <c r="Q7">
         <v>8.4</v>

</xml_diff>